<commit_message>
Updated filenames, Modified Test Data
</commit_message>
<xml_diff>
--- a/src/main/resources/edureka.xlsx
+++ b/src/main/resources/edureka.xlsx
@@ -1,40 +1,44 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
   <workbookPr defaultThemeVersion="166925"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:801_{BEB5E15B-877E-41F6-B40B-0D3647A53148}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\SeleniumWorkSpaceEclipse\edureka-automation-testing\src\main\resources\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E09361A7-E1FE-4D80-9FAD-21485AEA7A9A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{B61975A8-7105-4470-A3D6-068E94FB6268}"/>
+    <workbookView xWindow="720" yWindow="3225" windowWidth="17520" windowHeight="8655" firstSheet="8" activeTab="13" xr2:uid="{B61975A8-7105-4470-A3D6-068E94FB6268}"/>
   </bookViews>
   <sheets>
     <sheet name="SearchData" sheetId="1" r:id="rId1"/>
     <sheet name="Sheet1" sheetId="5" r:id="rId2"/>
-    <sheet name="AuthData" sheetId="2" r:id="rId3"/>
-    <sheet name="BlogData" sheetId="3" r:id="rId4"/>
-    <sheet name="CommunityQuestions" sheetId="4" r:id="rId5"/>
+    <sheet name="Professional" sheetId="6" r:id="rId3"/>
+    <sheet name="OtherDetails" sheetId="7" r:id="rId4"/>
+    <sheet name="Career" sheetId="8" r:id="rId5"/>
+    <sheet name="Topics" sheetId="9" r:id="rId6"/>
+    <sheet name="Personalize" sheetId="10" r:id="rId7"/>
+    <sheet name="LearningGoals" sheetId="11" r:id="rId8"/>
+    <sheet name="StudyPlan" sheetId="12" r:id="rId9"/>
+    <sheet name="InvalidData" sheetId="13" r:id="rId10"/>
+    <sheet name="AuthData" sheetId="2" r:id="rId11"/>
+    <sheet name="BlogData" sheetId="3" r:id="rId12"/>
+    <sheet name="CommunityQuestions" sheetId="4" r:id="rId13"/>
+    <sheet name="WebinarData" sheetId="14" r:id="rId14"/>
   </sheets>
   <calcPr calcId="0"/>
-  <oleSize ref="A1:O7"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="41">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="165" uniqueCount="146">
   <si>
     <t>email</t>
   </si>
@@ -157,13 +161,328 @@
   </si>
   <si>
     <t>test@gmail.com</t>
+  </si>
+  <si>
+    <t>companyName</t>
+  </si>
+  <si>
+    <t>linkedinURL</t>
+  </si>
+  <si>
+    <t>skills</t>
+  </si>
+  <si>
+    <t>jobLevel</t>
+  </si>
+  <si>
+    <t>currentIndustry</t>
+  </si>
+  <si>
+    <t>resumePath</t>
+  </si>
+  <si>
+    <t>TechCorp Solutions</t>
+  </si>
+  <si>
+    <t>https://linkedin.com/in/testuser</t>
+  </si>
+  <si>
+    <t>Java, Selenium</t>
+  </si>
+  <si>
+    <t>Senior Management</t>
+  </si>
+  <si>
+    <t>Insurance</t>
+  </si>
+  <si>
+    <t>C:\Users\RAMANA\Downloads\Infosys training material.pdf</t>
+  </si>
+  <si>
+    <t>DataSoft Inc</t>
+  </si>
+  <si>
+    <t>https://linkedin.com/in/user2</t>
+  </si>
+  <si>
+    <t>Python, SQL</t>
+  </si>
+  <si>
+    <t>Mid Management</t>
+  </si>
+  <si>
+    <t>IT-Software / Software Services</t>
+  </si>
+  <si>
+    <t>C:\Users\RAMANA\Downloads\shanmugam22.pdf</t>
+  </si>
+  <si>
+    <t>degree</t>
+  </si>
+  <si>
+    <t>institute</t>
+  </si>
+  <si>
+    <t>startMonth</t>
+  </si>
+  <si>
+    <t>startYear</t>
+  </si>
+  <si>
+    <t>endMonth</t>
+  </si>
+  <si>
+    <t>endYear</t>
+  </si>
+  <si>
+    <t>certName</t>
+  </si>
+  <si>
+    <t>certInstitute</t>
+  </si>
+  <si>
+    <t>B.Tech Computer</t>
+  </si>
+  <si>
+    <t>ABC College</t>
+  </si>
+  <si>
+    <t>June</t>
+  </si>
+  <si>
+    <t>2018</t>
+  </si>
+  <si>
+    <t>May</t>
+  </si>
+  <si>
+    <t>2022</t>
+  </si>
+  <si>
+    <t>Selenium Testing</t>
+  </si>
+  <si>
+    <t>Edureka</t>
+  </si>
+  <si>
+    <t>MBA</t>
+  </si>
+  <si>
+    <t>XYZ University</t>
+  </si>
+  <si>
+    <t>July</t>
+  </si>
+  <si>
+    <t>April</t>
+  </si>
+  <si>
+    <t>2024</t>
+  </si>
+  <si>
+    <t>Automation Cert</t>
+  </si>
+  <si>
+    <t>Udemy</t>
+  </si>
+  <si>
+    <t>interestedJob</t>
+  </si>
+  <si>
+    <t>employmentType</t>
+  </si>
+  <si>
+    <t>currentLocation</t>
+  </si>
+  <si>
+    <t>lastDrawnSalary</t>
+  </si>
+  <si>
+    <t>relocate</t>
+  </si>
+  <si>
+    <t>preferredLocation</t>
+  </si>
+  <si>
+    <t>Permanent</t>
+  </si>
+  <si>
+    <t>Bangalore</t>
+  </si>
+  <si>
+    <t>10-15 LPA</t>
+  </si>
+  <si>
+    <t>true</t>
+  </si>
+  <si>
+    <t>Hyderabad</t>
+  </si>
+  <si>
+    <t>Programming and Web Development</t>
+  </si>
+  <si>
+    <t>Contract</t>
+  </si>
+  <si>
+    <t>Chennai</t>
+  </si>
+  <si>
+    <t>5-10 LPA</t>
+  </si>
+  <si>
+    <t>false</t>
+  </si>
+  <si>
+    <t>topic1</t>
+  </si>
+  <si>
+    <t>topic2</t>
+  </si>
+  <si>
+    <t>topic3</t>
+  </si>
+  <si>
+    <t>Cloud Computing</t>
+  </si>
+  <si>
+    <t>Data Science</t>
+  </si>
+  <si>
+    <t>Python</t>
+  </si>
+  <si>
+    <t>Machine Learning</t>
+  </si>
+  <si>
+    <t>Cybersecurity</t>
+  </si>
+  <si>
+    <t>Java</t>
+  </si>
+  <si>
+    <t>Blockchain</t>
+  </si>
+  <si>
+    <t>Name</t>
+  </si>
+  <si>
+    <t>Designation</t>
+  </si>
+  <si>
+    <t>Industry</t>
+  </si>
+  <si>
+    <t>Experience</t>
+  </si>
+  <si>
+    <t>Timezone</t>
+  </si>
+  <si>
+    <t>PrefTimezone</t>
+  </si>
+  <si>
+    <t>WeekFrom</t>
+  </si>
+  <si>
+    <t>WeekTo</t>
+  </si>
+  <si>
+    <t>WeekendFrom</t>
+  </si>
+  <si>
+    <t>WeekendTo</t>
+  </si>
+  <si>
+    <t>Ram</t>
+  </si>
+  <si>
+    <t>QA Engineer</t>
+  </si>
+  <si>
+    <t>IT-Hardware &amp; Networking</t>
+  </si>
+  <si>
+    <t>0-2 years</t>
+  </si>
+  <si>
+    <t>India-IST-Asia/Kolkata</t>
+  </si>
+  <si>
+    <t>07:00 AM</t>
+  </si>
+  <si>
+    <t>08:00 AM</t>
+  </si>
+  <si>
+    <t>09:00 AM</t>
+  </si>
+  <si>
+    <t>10:00 AM</t>
+  </si>
+  <si>
+    <t>Goal</t>
+  </si>
+  <si>
+    <t>Higher Salary</t>
+  </si>
+  <si>
+    <t>Day</t>
+  </si>
+  <si>
+    <t>From</t>
+  </si>
+  <si>
+    <t>To</t>
+  </si>
+  <si>
+    <t>Friday</t>
+  </si>
+  <si>
+    <t>Saturday</t>
+  </si>
+  <si>
+    <t>Email</t>
+  </si>
+  <si>
+    <t>Phone</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sanjai </t>
+  </si>
+  <si>
+    <t>sanjai12345@email.com</t>
+  </si>
+  <si>
+    <t>Student</t>
+  </si>
+  <si>
+    <t>Kumar</t>
+  </si>
+  <si>
+    <t>kumar1234@gmail.com</t>
+  </si>
+  <si>
+    <t>Spiderman</t>
+  </si>
+  <si>
+    <t>spider12345@gmail.com</t>
+  </si>
+  <si>
+    <t>9078564534</t>
+  </si>
+  <si>
+    <t>8967564534</t>
+  </si>
+  <si>
+    <t>9067452378</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -187,16 +506,42 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF2E4057"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFEBF4F8"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -204,12 +549,27 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -224,6 +584,17 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -243,9 +614,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
-    <a:clrScheme name="Office 2013 - 2022">
+    <a:clrScheme name="Office">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -283,7 +654,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office 2013 - 2022">
+    <a:fontScheme name="Office">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -389,7 +760,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office 2013 - 2022">
+    <a:fmtScheme name="Office">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -531,7 +902,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -540,9 +911,9 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{111011FA-C08A-4F01-B9B7-9E860A471529}">
   <dimension ref="A1:G2"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>23</v>
       </c>
@@ -565,7 +936,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="2" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
         <v>30</v>
       </c>
@@ -593,12 +964,244 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{536B9051-A34A-4525-B37F-C21CC841DC31}">
+  <dimension ref="A1:A2"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>32</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E6343EBA-F3DC-423D-B377-70F5249FB146}">
+  <dimension ref="A1:B2"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="29" customWidth="1"/>
+    <col min="2" max="2" width="21.28515625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A2" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="A2" r:id="rId1" xr:uid="{D2F03319-B7BC-48ED-9A20-DAD8DCFA8694}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{33633261-1C6C-486C-BD2E-03EF2FD4779E}">
+  <dimension ref="A1:F2"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="15.42578125" customWidth="1"/>
+    <col min="2" max="2" width="15.28515625" customWidth="1"/>
+    <col min="3" max="3" width="16.7109375" customWidth="1"/>
+    <col min="4" max="4" width="15.7109375" customWidth="1"/>
+    <col min="5" max="5" width="18" customWidth="1"/>
+    <col min="6" max="6" width="16.28515625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A1" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" ht="60" x14ac:dyDescent="0.25">
+      <c r="A2" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="D2" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="E2" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="F2" s="3" t="s">
+        <v>15</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BA711BC9-A1D5-4B65-951C-7144E9AA05F5}">
+  <dimension ref="A1:D2"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="44" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="53.5703125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="4.5703125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>16</v>
+      </c>
+      <c r="B1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C1" t="s">
+        <v>17</v>
+      </c>
+      <c r="D1" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>19</v>
+      </c>
+      <c r="B2" t="s">
+        <v>20</v>
+      </c>
+      <c r="C2" t="s">
+        <v>21</v>
+      </c>
+      <c r="D2" t="s">
+        <v>22</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2C49F110-6CCC-47D5-9EE7-2893BAE7A162}">
+  <dimension ref="A1:D4"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="10.5703125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="23" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="11" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="10.85546875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1" s="9" t="s">
+        <v>108</v>
+      </c>
+      <c r="B1" s="9" t="s">
+        <v>134</v>
+      </c>
+      <c r="C1" s="9" t="s">
+        <v>135</v>
+      </c>
+      <c r="D1" s="9" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>136</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>137</v>
+      </c>
+      <c r="C2" s="10" t="s">
+        <v>143</v>
+      </c>
+      <c r="D2" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>139</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>140</v>
+      </c>
+      <c r="C3" s="10" t="s">
+        <v>144</v>
+      </c>
+      <c r="D3" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>141</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>142</v>
+      </c>
+      <c r="C4" s="10" t="s">
+        <v>145</v>
+      </c>
+      <c r="D4" t="s">
+        <v>138</v>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="B2" r:id="rId1" xr:uid="{5CA9A911-9151-48FB-95EE-B69EAB2AF309}"/>
+    <hyperlink ref="B3" r:id="rId2" xr:uid="{101D6A1C-C6FF-4574-9DFA-FCAE2DC8EBE4}"/>
+    <hyperlink ref="B4" r:id="rId3" xr:uid="{21862591-BB1E-44FD-BA5A-C73D88C1B429}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ED223D28-1E44-4A86-B887-6E90F2564441}">
   <dimension ref="A1:C2"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>37</v>
       </c>
@@ -609,7 +1212,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="2" spans="1:3" ht="72" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" ht="75" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
         <v>39</v>
       </c>
@@ -629,89 +1232,76 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E6343EBA-F3DC-423D-B377-70F5249FB146}">
-  <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E162EB23-E7C5-4092-A2DD-7A240E217818}">
+  <dimension ref="A1:F3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="29" customWidth="1"/>
-    <col min="2" max="2" width="21.21875" customWidth="1"/>
+    <col min="1" max="1" width="17.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="27.140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="13.5703125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="17.85546875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="27.140625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="51" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A2" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="B2" t="s">
-        <v>3</v>
-      </c>
-    </row>
-  </sheetData>
-  <hyperlinks>
-    <hyperlink ref="A2" r:id="rId1" xr:uid="{D2F03319-B7BC-48ED-9A20-DAD8DCFA8694}"/>
-  </hyperlinks>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{33633261-1C6C-486C-BD2E-03EF2FD4779E}">
-  <dimension ref="A1:F2"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <cols>
-    <col min="1" max="1" width="15.44140625" customWidth="1"/>
-    <col min="2" max="2" width="15.21875" customWidth="1"/>
-    <col min="3" max="3" width="16.77734375" customWidth="1"/>
-    <col min="4" max="4" width="15.77734375" customWidth="1"/>
-    <col min="5" max="5" width="18" customWidth="1"/>
-    <col min="6" max="6" width="16.21875" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A1" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="B1" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="D1" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="E1" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="F1" s="2" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="2" spans="1:6" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A2" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="B2" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="C2" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="D2" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="E2" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="F2" s="3" t="s">
-        <v>15</v>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A1" s="6" t="s">
+        <v>41</v>
+      </c>
+      <c r="B1" s="6" t="s">
+        <v>42</v>
+      </c>
+      <c r="C1" s="6" t="s">
+        <v>43</v>
+      </c>
+      <c r="D1" s="6" t="s">
+        <v>44</v>
+      </c>
+      <c r="E1" s="6" t="s">
+        <v>45</v>
+      </c>
+      <c r="F1" s="6" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A2" s="7" t="s">
+        <v>47</v>
+      </c>
+      <c r="B2" s="7" t="s">
+        <v>48</v>
+      </c>
+      <c r="C2" s="7" t="s">
+        <v>49</v>
+      </c>
+      <c r="D2" s="7" t="s">
+        <v>50</v>
+      </c>
+      <c r="E2" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="F2" s="7" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A3" s="8" t="s">
+        <v>53</v>
+      </c>
+      <c r="B3" s="8" t="s">
+        <v>54</v>
+      </c>
+      <c r="C3" s="8" t="s">
+        <v>55</v>
+      </c>
+      <c r="D3" s="8" t="s">
+        <v>56</v>
+      </c>
+      <c r="E3" s="8" t="s">
+        <v>57</v>
+      </c>
+      <c r="F3" s="8" t="s">
+        <v>58</v>
       </c>
     </row>
   </sheetData>
@@ -719,43 +1309,381 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BA711BC9-A1D5-4B65-951C-7144E9AA05F5}">
-  <dimension ref="A1:D2"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6E12843A-40AA-4FA4-BAA2-0F08EC8FB6CC}">
+  <dimension ref="A1:H3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="44" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="9.44140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="53.5546875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="4.5546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="16.28515625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.7109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10.85546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="8.85546875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="10.28515625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="8.28515625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="16.42578125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="12" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>16</v>
+        <v>59</v>
       </c>
       <c r="B1" t="s">
-        <v>7</v>
+        <v>60</v>
       </c>
       <c r="C1" t="s">
-        <v>17</v>
+        <v>61</v>
       </c>
       <c r="D1" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
+        <v>62</v>
+      </c>
+      <c r="E1" t="s">
+        <v>63</v>
+      </c>
+      <c r="F1" t="s">
+        <v>64</v>
+      </c>
+      <c r="G1" t="s">
+        <v>65</v>
+      </c>
+      <c r="H1" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>19</v>
+        <v>67</v>
       </c>
       <c r="B2" t="s">
-        <v>20</v>
+        <v>68</v>
       </c>
       <c r="C2" t="s">
-        <v>21</v>
+        <v>69</v>
       </c>
       <c r="D2" t="s">
-        <v>22</v>
+        <v>70</v>
+      </c>
+      <c r="E2" t="s">
+        <v>71</v>
+      </c>
+      <c r="F2" t="s">
+        <v>72</v>
+      </c>
+      <c r="G2" t="s">
+        <v>73</v>
+      </c>
+      <c r="H2" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>75</v>
+      </c>
+      <c r="B3" t="s">
+        <v>76</v>
+      </c>
+      <c r="C3" t="s">
+        <v>77</v>
+      </c>
+      <c r="D3" t="s">
+        <v>72</v>
+      </c>
+      <c r="E3" t="s">
+        <v>78</v>
+      </c>
+      <c r="F3" t="s">
+        <v>79</v>
+      </c>
+      <c r="G3" t="s">
+        <v>80</v>
+      </c>
+      <c r="H3" t="s">
+        <v>81</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5A257680-0D64-4E01-9920-015E40944413}">
+  <dimension ref="A1:F3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="31.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="18.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="4" width="17.42578125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="9.28515625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="19.7109375" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A1" s="6" t="s">
+        <v>82</v>
+      </c>
+      <c r="B1" s="6" t="s">
+        <v>83</v>
+      </c>
+      <c r="C1" s="6" t="s">
+        <v>84</v>
+      </c>
+      <c r="D1" s="6" t="s">
+        <v>85</v>
+      </c>
+      <c r="E1" s="6" t="s">
+        <v>86</v>
+      </c>
+      <c r="F1" s="6" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A2" s="7" t="s">
+        <v>34</v>
+      </c>
+      <c r="B2" s="7" t="s">
+        <v>88</v>
+      </c>
+      <c r="C2" s="7" t="s">
+        <v>89</v>
+      </c>
+      <c r="D2" s="7" t="s">
+        <v>90</v>
+      </c>
+      <c r="E2" s="7" t="s">
+        <v>91</v>
+      </c>
+      <c r="F2" s="7" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A3" s="8" t="s">
+        <v>93</v>
+      </c>
+      <c r="B3" s="8" t="s">
+        <v>94</v>
+      </c>
+      <c r="C3" s="8" t="s">
+        <v>95</v>
+      </c>
+      <c r="D3" s="8" t="s">
+        <v>96</v>
+      </c>
+      <c r="E3" s="8" t="s">
+        <v>97</v>
+      </c>
+      <c r="F3" s="8" t="s">
+        <v>95</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B9507B5E-862F-431D-8732-0E64AF54412E}">
+  <dimension ref="A1:C4"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="15.28515625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="15.7109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.42578125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A1" s="6" t="s">
+        <v>98</v>
+      </c>
+      <c r="B1" s="6" t="s">
+        <v>99</v>
+      </c>
+      <c r="C1" s="6" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2" s="7" t="s">
+        <v>101</v>
+      </c>
+      <c r="B2" s="7" t="s">
+        <v>102</v>
+      </c>
+      <c r="C2" s="7" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3" s="8" t="s">
+        <v>103</v>
+      </c>
+      <c r="B3" s="8" t="s">
+        <v>104</v>
+      </c>
+      <c r="C3" s="8" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A4" s="7" t="s">
+        <v>106</v>
+      </c>
+      <c r="B4" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="C4" s="7" t="s">
+        <v>107</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8507D311-0F24-4820-A0EB-5543FFCBFE08}">
+  <dimension ref="A1:J2"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="6.28515625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="12" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="25" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="10.85546875" bestFit="1" customWidth="1"/>
+    <col min="5" max="6" width="20.85546875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="10.7109375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="9" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="14.28515625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="11.7109375" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>108</v>
+      </c>
+      <c r="B1" t="s">
+        <v>109</v>
+      </c>
+      <c r="C1" t="s">
+        <v>110</v>
+      </c>
+      <c r="D1" t="s">
+        <v>111</v>
+      </c>
+      <c r="E1" t="s">
+        <v>112</v>
+      </c>
+      <c r="F1" t="s">
+        <v>113</v>
+      </c>
+      <c r="G1" t="s">
+        <v>114</v>
+      </c>
+      <c r="H1" t="s">
+        <v>115</v>
+      </c>
+      <c r="I1" t="s">
+        <v>116</v>
+      </c>
+      <c r="J1" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>118</v>
+      </c>
+      <c r="B2" t="s">
+        <v>119</v>
+      </c>
+      <c r="C2" t="s">
+        <v>120</v>
+      </c>
+      <c r="D2" t="s">
+        <v>121</v>
+      </c>
+      <c r="E2" t="s">
+        <v>122</v>
+      </c>
+      <c r="F2" t="s">
+        <v>122</v>
+      </c>
+      <c r="G2" t="s">
+        <v>123</v>
+      </c>
+      <c r="H2" t="s">
+        <v>124</v>
+      </c>
+      <c r="I2" t="s">
+        <v>125</v>
+      </c>
+      <c r="J2" t="s">
+        <v>126</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B3B887BA-2813-4CE1-A1C9-16150E464297}">
+  <dimension ref="A1:A2"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>128</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FD50E61C-6B07-4FD3-A611-B3A1E8E55C1D}">
+  <dimension ref="A1:C3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>129</v>
+      </c>
+      <c r="B1" t="s">
+        <v>130</v>
+      </c>
+      <c r="C1" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>132</v>
+      </c>
+      <c r="B2" t="s">
+        <v>123</v>
+      </c>
+      <c r="C2" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>133</v>
+      </c>
+      <c r="B3" t="s">
+        <v>124</v>
+      </c>
+      <c r="C3" t="s">
+        <v>125</v>
       </c>
     </row>
   </sheetData>

</xml_diff>